<commit_message>
[FIX] Invoice with RC
</commit_message>
<xml_diff>
--- a/l10n_it_reverse_charge/tests/data/account_fiscal_position.xlsx
+++ b/l10n_it_reverse_charge/tests/data/account_fiscal_position.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="36">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -43,6 +43,24 @@
     <t xml:space="preserve">rc_type_id</t>
   </si>
   <si>
+    <t xml:space="preserve">rc_type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">partner_type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">self_journal_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">payment_journal_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">transient_account_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rc_fiscal_document_type_id</t>
+  </si>
+  <si>
     <t xml:space="preserve">z0bug.fiscalpos_it</t>
   </si>
   <si>
@@ -58,6 +76,24 @@
     <t xml:space="preserve">l10n_it_reverse_charge.account_rc_type_1</t>
   </si>
   <si>
+    <t xml:space="preserve">self</t>
+  </si>
+  <si>
+    <t xml:space="preserve">supplier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">external.INV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">z0bug.jou_gc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">z0bug.coa_gc_rc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">external.TD19</t>
+  </si>
+  <si>
     <t xml:space="preserve">z0bug.fiscalpos_eu</t>
   </si>
   <si>
@@ -67,6 +103,9 @@
     <t xml:space="preserve">l10n_it_reverse_charge.account_rc_type_2</t>
   </si>
   <si>
+    <t xml:space="preserve">external.TD18</t>
+  </si>
+  <si>
     <t xml:space="preserve">z0bug.fiscalpos_xx</t>
   </si>
   <si>
@@ -74,6 +113,12 @@
   </si>
   <si>
     <t xml:space="preserve">l10n_it_reverse_charge.account_rc_type_3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">other</t>
+  </si>
+  <si>
+    <t xml:space="preserve">external.TD17</t>
   </si>
   <si>
     <t xml:space="preserve">z0bug.fiscalpos_sp</t>
@@ -93,7 +138,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -114,6 +159,13 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -158,12 +210,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -294,7 +354,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16.17"/>
@@ -304,6 +364,11 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12.84"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="26.32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="36.06"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="7.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="13.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="17.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="18.26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="21.6"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -328,72 +393,150 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>8</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>8</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>11</v>
+        <v>17</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="M3" s="3" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>12</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>14</v>
+        <v>26</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="M4" s="3" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>16</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>17</v>
+        <v>30</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="M5" s="3" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>20</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>20</v>
+        <v>34</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>